<commit_message>
Update supplementary materials to v13
- Fix d_i for T1578.002 (Update server) in scenario A (5 -> 3); recomputed results
- Add sensitivity_extra.py (Ci/Pi uniform and Monte Carlo per-step Pi +-5%) and results
- Add check_di_consistency.py and results/di_consistency.csv
- README: F_k=0 sub-technique Level-1 note, change log
</commit_message>
<xml_diff>
--- a/SPRV/SPRV_LG_LONG_scenarioA.xlsx
+++ b/SPRV/SPRV_LG_LONG_scenarioA.xlsx
@@ -1303,7 +1303,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AC257"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14"/>
@@ -15246,22 +15246,22 @@
         <v>0.36</v>
       </c>
       <c r="J131" s="4" t="n">
-        <v>0.1</v>
+        <v>0.46</v>
       </c>
       <c r="K131" s="4" t="n">
         <v>1.5</v>
       </c>
       <c r="L131" s="4" t="n">
         <f aca="false">I131*J131</f>
-        <v>0.036</v>
+        <v>0.1656</v>
       </c>
       <c r="M131" s="4" t="n">
         <f aca="false">MIN(1,I131*J131*K131)</f>
-        <v>0.054</v>
+        <v>0.2484</v>
       </c>
       <c r="N131" s="4" t="n">
         <f aca="false">N130*M131</f>
-        <v>0.007776</v>
+        <v>0.0357696</v>
       </c>
       <c r="O131" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -15313,7 +15313,7 @@
       </c>
       <c r="AA131" s="3" t="n">
         <f aca="false">IF(J131&gt;='Settings '!$B$10,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB131" s="3" t="n">
         <f aca="false">IF(M131&gt;='Settings '!$B$11,1,0)</f>
@@ -15368,7 +15368,7 @@
       </c>
       <c r="N132" s="4" t="n">
         <f aca="false">N131*M132</f>
-        <v>0.000559872</v>
+        <v>0.0025754112</v>
       </c>
       <c r="O132" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -15475,7 +15475,7 @@
       </c>
       <c r="N133" s="4" t="n">
         <f aca="false">N132*M133</f>
-        <v>0.00010077696</v>
+        <v>0.000463574016</v>
       </c>
       <c r="O133" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -15503,7 +15503,7 @@
       </c>
       <c r="U133" s="4" t="n">
         <f aca="false">IF(E133=4,N133,"")</f>
-        <v>0.00010077696</v>
+        <v>0.000463574016</v>
       </c>
       <c r="V133" s="4" t="n">
         <f aca="false">IF(E133=4,Q133,"")</f>
@@ -15515,7 +15515,7 @@
       </c>
       <c r="X133" s="4" t="n">
         <f aca="false">IF(E133=4,IFERROR((LN(U133)-LN(V133))/(LN(W133)-LN(V133)),0),"")</f>
-        <v>0</v>
+        <v>0.189638418693276</v>
       </c>
       <c r="Y133" s="3" t="str">
         <f aca="false">IF(E133=4,IF(X133&gt;='Settings '!$B$7,"Risk A",IF(X133&gt;='Settings '!$B$6,"Risk B","Risk C")),"")</f>
@@ -15674,22 +15674,22 @@
         <v>0.36</v>
       </c>
       <c r="J135" s="4" t="n">
-        <v>0.1</v>
+        <v>0.46</v>
       </c>
       <c r="K135" s="4" t="n">
         <v>1.5</v>
       </c>
       <c r="L135" s="4" t="n">
         <f aca="false">I135*J135</f>
-        <v>0.036</v>
+        <v>0.1656</v>
       </c>
       <c r="M135" s="4" t="n">
         <f aca="false">MIN(1,I135*J135*K135)</f>
-        <v>0.054</v>
+        <v>0.2484</v>
       </c>
       <c r="N135" s="4" t="n">
         <f aca="false">N134*M135</f>
-        <v>0.007776</v>
+        <v>0.0357696</v>
       </c>
       <c r="O135" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -15741,7 +15741,7 @@
       </c>
       <c r="AA135" s="3" t="n">
         <f aca="false">IF(J135&gt;='Settings '!$B$10,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB135" s="3" t="n">
         <f aca="false">IF(M135&gt;='Settings '!$B$11,1,0)</f>
@@ -15796,7 +15796,7 @@
       </c>
       <c r="N136" s="4" t="n">
         <f aca="false">N135*M136</f>
-        <v>0.000559872</v>
+        <v>0.0025754112</v>
       </c>
       <c r="O136" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -15903,7 +15903,7 @@
       </c>
       <c r="N137" s="4" t="n">
         <f aca="false">N136*M137</f>
-        <v>0.0002257403904</v>
+        <v>0.00103840579584</v>
       </c>
       <c r="O137" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -15931,7 +15931,7 @@
       </c>
       <c r="U137" s="4" t="n">
         <f aca="false">IF(E137=4,N137,"")</f>
-        <v>0.0002257403904</v>
+        <v>0.00103840579584</v>
       </c>
       <c r="V137" s="4" t="n">
         <f aca="false">IF(E137=4,Q137,"")</f>
@@ -15943,7 +15943,7 @@
       </c>
       <c r="X137" s="4" t="n">
         <f aca="false">IF(E137=4,IFERROR((LN(U137)-LN(V137))/(LN(W137)-LN(V137)),0),"")</f>
-        <v>0.124495519473378</v>
+        <v>0.309017265158183</v>
       </c>
       <c r="Y137" s="3" t="str">
         <f aca="false">IF(E137=4,IF(X137&gt;='Settings '!$B$7,"Risk A",IF(X137&gt;='Settings '!$B$6,"Risk B","Risk C")),"")</f>
@@ -16102,22 +16102,22 @@
         <v>0.36</v>
       </c>
       <c r="J139" s="4" t="n">
-        <v>0.1</v>
+        <v>0.46</v>
       </c>
       <c r="K139" s="4" t="n">
         <v>1.5</v>
       </c>
       <c r="L139" s="4" t="n">
         <f aca="false">I139*J139</f>
-        <v>0.036</v>
+        <v>0.1656</v>
       </c>
       <c r="M139" s="4" t="n">
         <f aca="false">MIN(1,I139*J139*K139)</f>
-        <v>0.054</v>
+        <v>0.2484</v>
       </c>
       <c r="N139" s="4" t="n">
         <f aca="false">N138*M139</f>
-        <v>0.007776</v>
+        <v>0.0357696</v>
       </c>
       <c r="O139" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -16169,7 +16169,7 @@
       </c>
       <c r="AA139" s="3" t="n">
         <f aca="false">IF(J139&gt;='Settings '!$B$10,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB139" s="3" t="n">
         <f aca="false">IF(M139&gt;='Settings '!$B$11,1,0)</f>
@@ -16224,7 +16224,7 @@
       </c>
       <c r="N140" s="4" t="n">
         <f aca="false">N139*M140</f>
-        <v>0.000559872</v>
+        <v>0.0025754112</v>
       </c>
       <c r="O140" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -16331,7 +16331,7 @@
       </c>
       <c r="N141" s="4" t="n">
         <f aca="false">N140*M141</f>
-        <v>5.64350976E-005</v>
+        <v>0.00025960144896</v>
       </c>
       <c r="O141" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -16359,7 +16359,7 @@
       </c>
       <c r="U141" s="4" t="n">
         <f aca="false">IF(E141=4,N141,"")</f>
-        <v>5.64350976E-005</v>
+        <v>0.00025960144896</v>
       </c>
       <c r="V141" s="4" t="n">
         <f aca="false">IF(E141=4,Q141,"")</f>
@@ -16371,7 +16371,7 @@
       </c>
       <c r="X141" s="4" t="n">
         <f aca="false">IF(E141=4,IFERROR((LN(U141)-LN(V141))/(LN(W141)-LN(V141)),0),"")</f>
-        <v>0.120711114312368</v>
+        <v>0.29962378225974</v>
       </c>
       <c r="Y141" s="3" t="str">
         <f aca="false">IF(E141=4,IF(X141&gt;='Settings '!$B$7,"Risk A",IF(X141&gt;='Settings '!$B$6,"Risk B","Risk C")),"")</f>
@@ -16530,22 +16530,22 @@
         <v>0.36</v>
       </c>
       <c r="J143" s="4" t="n">
-        <v>0.1</v>
+        <v>0.46</v>
       </c>
       <c r="K143" s="4" t="n">
         <v>1.5</v>
       </c>
       <c r="L143" s="4" t="n">
         <f aca="false">I143*J143</f>
-        <v>0.036</v>
+        <v>0.1656</v>
       </c>
       <c r="M143" s="4" t="n">
         <f aca="false">MIN(1,I143*J143*K143)</f>
-        <v>0.054</v>
+        <v>0.2484</v>
       </c>
       <c r="N143" s="4" t="n">
         <f aca="false">N142*M143</f>
-        <v>0.007776</v>
+        <v>0.0357696</v>
       </c>
       <c r="O143" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -16597,7 +16597,7 @@
       </c>
       <c r="AA143" s="3" t="n">
         <f aca="false">IF(J143&gt;='Settings '!$B$10,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB143" s="3" t="n">
         <f aca="false">IF(M143&gt;='Settings '!$B$11,1,0)</f>
@@ -16652,7 +16652,7 @@
       </c>
       <c r="N144" s="4" t="n">
         <f aca="false">N143*M144</f>
-        <v>0.000559872</v>
+        <v>0.0025754112</v>
       </c>
       <c r="O144" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -16759,7 +16759,7 @@
       </c>
       <c r="N145" s="4" t="n">
         <f aca="false">N144*M145</f>
-        <v>5.64350976E-005</v>
+        <v>0.00025960144896</v>
       </c>
       <c r="O145" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -16787,7 +16787,7 @@
       </c>
       <c r="U145" s="4" t="n">
         <f aca="false">IF(E145=4,N145,"")</f>
-        <v>5.64350976E-005</v>
+        <v>0.00025960144896</v>
       </c>
       <c r="V145" s="4" t="n">
         <f aca="false">IF(E145=4,Q145,"")</f>
@@ -16799,7 +16799,7 @@
       </c>
       <c r="X145" s="4" t="n">
         <f aca="false">IF(E145=4,IFERROR((LN(U145)-LN(V145))/(LN(W145)-LN(V145)),0),"")</f>
-        <v>0.120711114312368</v>
+        <v>0.29962378225974</v>
       </c>
       <c r="Y145" s="3" t="str">
         <f aca="false">IF(E145=4,IF(X145&gt;='Settings '!$B$7,"Risk A",IF(X145&gt;='Settings '!$B$6,"Risk B","Risk C")),"")</f>
@@ -16958,22 +16958,22 @@
         <v>0.36</v>
       </c>
       <c r="J147" s="4" t="n">
-        <v>0.1</v>
+        <v>0.46</v>
       </c>
       <c r="K147" s="4" t="n">
         <v>1.5</v>
       </c>
       <c r="L147" s="4" t="n">
         <f aca="false">I147*J147</f>
-        <v>0.036</v>
+        <v>0.1656</v>
       </c>
       <c r="M147" s="4" t="n">
         <f aca="false">MIN(1,I147*J147*K147)</f>
-        <v>0.054</v>
+        <v>0.2484</v>
       </c>
       <c r="N147" s="4" t="n">
         <f aca="false">N146*M147</f>
-        <v>0.007776</v>
+        <v>0.0357696</v>
       </c>
       <c r="O147" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -17025,7 +17025,7 @@
       </c>
       <c r="AA147" s="3" t="n">
         <f aca="false">IF(J147&gt;='Settings '!$B$10,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB147" s="3" t="n">
         <f aca="false">IF(M147&gt;='Settings '!$B$11,1,0)</f>
@@ -17080,7 +17080,7 @@
       </c>
       <c r="N148" s="4" t="n">
         <f aca="false">N147*M148</f>
-        <v>0.000559872</v>
+        <v>0.0025754112</v>
       </c>
       <c r="O148" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -17187,7 +17187,7 @@
       </c>
       <c r="N149" s="4" t="n">
         <f aca="false">N148*M149</f>
-        <v>0.00010077696</v>
+        <v>0.000463574016</v>
       </c>
       <c r="O149" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -17215,7 +17215,7 @@
       </c>
       <c r="U149" s="4" t="n">
         <f aca="false">IF(E149=4,N149,"")</f>
-        <v>0.00010077696</v>
+        <v>0.000463574016</v>
       </c>
       <c r="V149" s="4" t="n">
         <f aca="false">IF(E149=4,Q149,"")</f>
@@ -17227,7 +17227,7 @@
       </c>
       <c r="X149" s="4" t="n">
         <f aca="false">IF(E149=4,IFERROR((LN(U149)-LN(V149))/(LN(W149)-LN(V149)),0),"")</f>
-        <v>0</v>
+        <v>0.189638418693276</v>
       </c>
       <c r="Y149" s="3" t="str">
         <f aca="false">IF(E149=4,IF(X149&gt;='Settings '!$B$7,"Risk A",IF(X149&gt;='Settings '!$B$6,"Risk B","Risk C")),"")</f>
@@ -17386,22 +17386,22 @@
         <v>0.36</v>
       </c>
       <c r="J151" s="4" t="n">
-        <v>0.1</v>
+        <v>0.46</v>
       </c>
       <c r="K151" s="4" t="n">
         <v>1.5</v>
       </c>
       <c r="L151" s="4" t="n">
         <f aca="false">I151*J151</f>
-        <v>0.036</v>
+        <v>0.1656</v>
       </c>
       <c r="M151" s="4" t="n">
         <f aca="false">MIN(1,I151*J151*K151)</f>
-        <v>0.054</v>
+        <v>0.2484</v>
       </c>
       <c r="N151" s="4" t="n">
         <f aca="false">N150*M151</f>
-        <v>0.007776</v>
+        <v>0.0357696</v>
       </c>
       <c r="O151" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -17453,7 +17453,7 @@
       </c>
       <c r="AA151" s="3" t="n">
         <f aca="false">IF(J151&gt;='Settings '!$B$10,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB151" s="3" t="n">
         <f aca="false">IF(M151&gt;='Settings '!$B$11,1,0)</f>
@@ -17508,7 +17508,7 @@
       </c>
       <c r="N152" s="4" t="n">
         <f aca="false">N151*M152</f>
-        <v>0.000559872</v>
+        <v>0.0025754112</v>
       </c>
       <c r="O152" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -17615,7 +17615,7 @@
       </c>
       <c r="N153" s="4" t="n">
         <f aca="false">N152*M153</f>
-        <v>0.0002257403904</v>
+        <v>0.00103840579584</v>
       </c>
       <c r="O153" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -17643,7 +17643,7 @@
       </c>
       <c r="U153" s="4" t="n">
         <f aca="false">IF(E153=4,N153,"")</f>
-        <v>0.0002257403904</v>
+        <v>0.00103840579584</v>
       </c>
       <c r="V153" s="4" t="n">
         <f aca="false">IF(E153=4,Q153,"")</f>
@@ -17655,7 +17655,7 @@
       </c>
       <c r="X153" s="4" t="n">
         <f aca="false">IF(E153=4,IFERROR((LN(U153)-LN(V153))/(LN(W153)-LN(V153)),0),"")</f>
-        <v>0.124495519473378</v>
+        <v>0.309017265158183</v>
       </c>
       <c r="Y153" s="3" t="str">
         <f aca="false">IF(E153=4,IF(X153&gt;='Settings '!$B$7,"Risk A",IF(X153&gt;='Settings '!$B$6,"Risk B","Risk C")),"")</f>
@@ -17814,22 +17814,22 @@
         <v>0.36</v>
       </c>
       <c r="J155" s="4" t="n">
-        <v>0.1</v>
+        <v>0.46</v>
       </c>
       <c r="K155" s="4" t="n">
         <v>1.5</v>
       </c>
       <c r="L155" s="4" t="n">
         <f aca="false">I155*J155</f>
-        <v>0.036</v>
+        <v>0.1656</v>
       </c>
       <c r="M155" s="4" t="n">
         <f aca="false">MIN(1,I155*J155*K155)</f>
-        <v>0.054</v>
+        <v>0.2484</v>
       </c>
       <c r="N155" s="4" t="n">
         <f aca="false">N154*M155</f>
-        <v>0.007776</v>
+        <v>0.0357696</v>
       </c>
       <c r="O155" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -17881,7 +17881,7 @@
       </c>
       <c r="AA155" s="3" t="n">
         <f aca="false">IF(J155&gt;='Settings '!$B$10,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB155" s="3" t="n">
         <f aca="false">IF(M155&gt;='Settings '!$B$11,1,0)</f>
@@ -17936,7 +17936,7 @@
       </c>
       <c r="N156" s="4" t="n">
         <f aca="false">N155*M156</f>
-        <v>0.000559872</v>
+        <v>0.0025754112</v>
       </c>
       <c r="O156" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -18043,7 +18043,7 @@
       </c>
       <c r="N157" s="4" t="n">
         <f aca="false">N156*M157</f>
-        <v>5.64350976E-005</v>
+        <v>0.00025960144896</v>
       </c>
       <c r="O157" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -18071,7 +18071,7 @@
       </c>
       <c r="U157" s="4" t="n">
         <f aca="false">IF(E157=4,N157,"")</f>
-        <v>5.64350976E-005</v>
+        <v>0.00025960144896</v>
       </c>
       <c r="V157" s="4" t="n">
         <f aca="false">IF(E157=4,Q157,"")</f>
@@ -18083,7 +18083,7 @@
       </c>
       <c r="X157" s="4" t="n">
         <f aca="false">IF(E157=4,IFERROR((LN(U157)-LN(V157))/(LN(W157)-LN(V157)),0),"")</f>
-        <v>0.120711114312368</v>
+        <v>0.29962378225974</v>
       </c>
       <c r="Y157" s="3" t="str">
         <f aca="false">IF(E157=4,IF(X157&gt;='Settings '!$B$7,"Risk A",IF(X157&gt;='Settings '!$B$6,"Risk B","Risk C")),"")</f>
@@ -18242,22 +18242,22 @@
         <v>0.36</v>
       </c>
       <c r="J159" s="4" t="n">
-        <v>0.1</v>
+        <v>0.46</v>
       </c>
       <c r="K159" s="4" t="n">
         <v>1.5</v>
       </c>
       <c r="L159" s="4" t="n">
         <f aca="false">I159*J159</f>
-        <v>0.036</v>
+        <v>0.1656</v>
       </c>
       <c r="M159" s="4" t="n">
         <f aca="false">MIN(1,I159*J159*K159)</f>
-        <v>0.054</v>
+        <v>0.2484</v>
       </c>
       <c r="N159" s="4" t="n">
         <f aca="false">N158*M159</f>
-        <v>0.007776</v>
+        <v>0.0357696</v>
       </c>
       <c r="O159" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -18309,7 +18309,7 @@
       </c>
       <c r="AA159" s="3" t="n">
         <f aca="false">IF(J159&gt;='Settings '!$B$10,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB159" s="3" t="n">
         <f aca="false">IF(M159&gt;='Settings '!$B$11,1,0)</f>
@@ -18364,7 +18364,7 @@
       </c>
       <c r="N160" s="4" t="n">
         <f aca="false">N159*M160</f>
-        <v>0.000559872</v>
+        <v>0.0025754112</v>
       </c>
       <c r="O160" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -18471,7 +18471,7 @@
       </c>
       <c r="N161" s="4" t="n">
         <f aca="false">N160*M161</f>
-        <v>5.64350976E-005</v>
+        <v>0.00025960144896</v>
       </c>
       <c r="O161" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -18499,7 +18499,7 @@
       </c>
       <c r="U161" s="4" t="n">
         <f aca="false">IF(E161=4,N161,"")</f>
-        <v>5.64350976E-005</v>
+        <v>0.00025960144896</v>
       </c>
       <c r="V161" s="4" t="n">
         <f aca="false">IF(E161=4,Q161,"")</f>
@@ -18511,7 +18511,7 @@
       </c>
       <c r="X161" s="4" t="n">
         <f aca="false">IF(E161=4,IFERROR((LN(U161)-LN(V161))/(LN(W161)-LN(V161)),0),"")</f>
-        <v>0.120711114312368</v>
+        <v>0.29962378225974</v>
       </c>
       <c r="Y161" s="3" t="str">
         <f aca="false">IF(E161=4,IF(X161&gt;='Settings '!$B$7,"Risk A",IF(X161&gt;='Settings '!$B$6,"Risk B","Risk C")),"")</f>
@@ -18670,22 +18670,22 @@
         <v>0.36</v>
       </c>
       <c r="J163" s="4" t="n">
-        <v>0.1</v>
+        <v>0.46</v>
       </c>
       <c r="K163" s="4" t="n">
         <v>1.5</v>
       </c>
       <c r="L163" s="4" t="n">
         <f aca="false">I163*J163</f>
-        <v>0.036</v>
+        <v>0.1656</v>
       </c>
       <c r="M163" s="4" t="n">
         <f aca="false">MIN(1,I163*J163*K163)</f>
-        <v>0.054</v>
+        <v>0.2484</v>
       </c>
       <c r="N163" s="4" t="n">
         <f aca="false">N162*M163</f>
-        <v>0.007776</v>
+        <v>0.0357696</v>
       </c>
       <c r="O163" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -18737,7 +18737,7 @@
       </c>
       <c r="AA163" s="3" t="n">
         <f aca="false">IF(J163&gt;='Settings '!$B$10,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB163" s="3" t="n">
         <f aca="false">IF(M163&gt;='Settings '!$B$11,1,0)</f>
@@ -18792,7 +18792,7 @@
       </c>
       <c r="N164" s="4" t="n">
         <f aca="false">N163*M164</f>
-        <v>0.000559872</v>
+        <v>0.0025754112</v>
       </c>
       <c r="O164" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -18899,7 +18899,7 @@
       </c>
       <c r="N165" s="4" t="n">
         <f aca="false">N164*M165</f>
-        <v>0.00010077696</v>
+        <v>0.000463574016</v>
       </c>
       <c r="O165" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -18927,7 +18927,7 @@
       </c>
       <c r="U165" s="4" t="n">
         <f aca="false">IF(E165=4,N165,"")</f>
-        <v>0.00010077696</v>
+        <v>0.000463574016</v>
       </c>
       <c r="V165" s="4" t="n">
         <f aca="false">IF(E165=4,Q165,"")</f>
@@ -18939,7 +18939,7 @@
       </c>
       <c r="X165" s="4" t="n">
         <f aca="false">IF(E165=4,IFERROR((LN(U165)-LN(V165))/(LN(W165)-LN(V165)),0),"")</f>
-        <v>0</v>
+        <v>0.189638418693276</v>
       </c>
       <c r="Y165" s="3" t="str">
         <f aca="false">IF(E165=4,IF(X165&gt;='Settings '!$B$7,"Risk A",IF(X165&gt;='Settings '!$B$6,"Risk B","Risk C")),"")</f>
@@ -19098,22 +19098,22 @@
         <v>0.36</v>
       </c>
       <c r="J167" s="4" t="n">
-        <v>0.1</v>
+        <v>0.46</v>
       </c>
       <c r="K167" s="4" t="n">
         <v>1.5</v>
       </c>
       <c r="L167" s="4" t="n">
         <f aca="false">I167*J167</f>
-        <v>0.036</v>
+        <v>0.1656</v>
       </c>
       <c r="M167" s="4" t="n">
         <f aca="false">MIN(1,I167*J167*K167)</f>
-        <v>0.054</v>
+        <v>0.2484</v>
       </c>
       <c r="N167" s="4" t="n">
         <f aca="false">N166*M167</f>
-        <v>0.007776</v>
+        <v>0.0357696</v>
       </c>
       <c r="O167" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -19165,7 +19165,7 @@
       </c>
       <c r="AA167" s="3" t="n">
         <f aca="false">IF(J167&gt;='Settings '!$B$10,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB167" s="3" t="n">
         <f aca="false">IF(M167&gt;='Settings '!$B$11,1,0)</f>
@@ -19220,7 +19220,7 @@
       </c>
       <c r="N168" s="4" t="n">
         <f aca="false">N167*M168</f>
-        <v>0.000559872</v>
+        <v>0.0025754112</v>
       </c>
       <c r="O168" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -19327,7 +19327,7 @@
       </c>
       <c r="N169" s="4" t="n">
         <f aca="false">N168*M169</f>
-        <v>0.0002257403904</v>
+        <v>0.00103840579584</v>
       </c>
       <c r="O169" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -19355,7 +19355,7 @@
       </c>
       <c r="U169" s="4" t="n">
         <f aca="false">IF(E169=4,N169,"")</f>
-        <v>0.0002257403904</v>
+        <v>0.00103840579584</v>
       </c>
       <c r="V169" s="4" t="n">
         <f aca="false">IF(E169=4,Q169,"")</f>
@@ -19367,7 +19367,7 @@
       </c>
       <c r="X169" s="4" t="n">
         <f aca="false">IF(E169=4,IFERROR((LN(U169)-LN(V169))/(LN(W169)-LN(V169)),0),"")</f>
-        <v>0.124495519473378</v>
+        <v>0.309017265158183</v>
       </c>
       <c r="Y169" s="3" t="str">
         <f aca="false">IF(E169=4,IF(X169&gt;='Settings '!$B$7,"Risk A",IF(X169&gt;='Settings '!$B$6,"Risk B","Risk C")),"")</f>
@@ -19526,22 +19526,22 @@
         <v>0.36</v>
       </c>
       <c r="J171" s="4" t="n">
-        <v>0.1</v>
+        <v>0.46</v>
       </c>
       <c r="K171" s="4" t="n">
         <v>1.5</v>
       </c>
       <c r="L171" s="4" t="n">
         <f aca="false">I171*J171</f>
-        <v>0.036</v>
+        <v>0.1656</v>
       </c>
       <c r="M171" s="4" t="n">
         <f aca="false">MIN(1,I171*J171*K171)</f>
-        <v>0.054</v>
+        <v>0.2484</v>
       </c>
       <c r="N171" s="4" t="n">
         <f aca="false">N170*M171</f>
-        <v>0.007776</v>
+        <v>0.0357696</v>
       </c>
       <c r="O171" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -19593,7 +19593,7 @@
       </c>
       <c r="AA171" s="3" t="n">
         <f aca="false">IF(J171&gt;='Settings '!$B$10,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB171" s="3" t="n">
         <f aca="false">IF(M171&gt;='Settings '!$B$11,1,0)</f>
@@ -19648,7 +19648,7 @@
       </c>
       <c r="N172" s="4" t="n">
         <f aca="false">N171*M172</f>
-        <v>0.000559872</v>
+        <v>0.0025754112</v>
       </c>
       <c r="O172" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -19755,7 +19755,7 @@
       </c>
       <c r="N173" s="4" t="n">
         <f aca="false">N172*M173</f>
-        <v>5.64350976E-005</v>
+        <v>0.00025960144896</v>
       </c>
       <c r="O173" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -19783,7 +19783,7 @@
       </c>
       <c r="U173" s="4" t="n">
         <f aca="false">IF(E173=4,N173,"")</f>
-        <v>5.64350976E-005</v>
+        <v>0.00025960144896</v>
       </c>
       <c r="V173" s="4" t="n">
         <f aca="false">IF(E173=4,Q173,"")</f>
@@ -19795,7 +19795,7 @@
       </c>
       <c r="X173" s="4" t="n">
         <f aca="false">IF(E173=4,IFERROR((LN(U173)-LN(V173))/(LN(W173)-LN(V173)),0),"")</f>
-        <v>0.120711114312368</v>
+        <v>0.29962378225974</v>
       </c>
       <c r="Y173" s="3" t="str">
         <f aca="false">IF(E173=4,IF(X173&gt;='Settings '!$B$7,"Risk A",IF(X173&gt;='Settings '!$B$6,"Risk B","Risk C")),"")</f>
@@ -19954,22 +19954,22 @@
         <v>0.36</v>
       </c>
       <c r="J175" s="4" t="n">
-        <v>0.1</v>
+        <v>0.46</v>
       </c>
       <c r="K175" s="4" t="n">
         <v>1.5</v>
       </c>
       <c r="L175" s="4" t="n">
         <f aca="false">I175*J175</f>
-        <v>0.036</v>
+        <v>0.1656</v>
       </c>
       <c r="M175" s="4" t="n">
         <f aca="false">MIN(1,I175*J175*K175)</f>
-        <v>0.054</v>
+        <v>0.2484</v>
       </c>
       <c r="N175" s="4" t="n">
         <f aca="false">N174*M175</f>
-        <v>0.007776</v>
+        <v>0.0357696</v>
       </c>
       <c r="O175" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -20021,7 +20021,7 @@
       </c>
       <c r="AA175" s="3" t="n">
         <f aca="false">IF(J175&gt;='Settings '!$B$10,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB175" s="3" t="n">
         <f aca="false">IF(M175&gt;='Settings '!$B$11,1,0)</f>
@@ -20076,7 +20076,7 @@
       </c>
       <c r="N176" s="4" t="n">
         <f aca="false">N175*M176</f>
-        <v>0.000559872</v>
+        <v>0.0025754112</v>
       </c>
       <c r="O176" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -20183,7 +20183,7 @@
       </c>
       <c r="N177" s="4" t="n">
         <f aca="false">N176*M177</f>
-        <v>5.64350976E-005</v>
+        <v>0.00025960144896</v>
       </c>
       <c r="O177" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -20211,7 +20211,7 @@
       </c>
       <c r="U177" s="4" t="n">
         <f aca="false">IF(E177=4,N177,"")</f>
-        <v>5.64350976E-005</v>
+        <v>0.00025960144896</v>
       </c>
       <c r="V177" s="4" t="n">
         <f aca="false">IF(E177=4,Q177,"")</f>
@@ -20223,7 +20223,7 @@
       </c>
       <c r="X177" s="4" t="n">
         <f aca="false">IF(E177=4,IFERROR((LN(U177)-LN(V177))/(LN(W177)-LN(V177)),0),"")</f>
-        <v>0.120711114312368</v>
+        <v>0.29962378225974</v>
       </c>
       <c r="Y177" s="3" t="str">
         <f aca="false">IF(E177=4,IF(X177&gt;='Settings '!$B$7,"Risk A",IF(X177&gt;='Settings '!$B$6,"Risk B","Risk C")),"")</f>
@@ -20382,22 +20382,22 @@
         <v>0.36</v>
       </c>
       <c r="J179" s="4" t="n">
-        <v>0.1</v>
+        <v>0.46</v>
       </c>
       <c r="K179" s="4" t="n">
         <v>1.5</v>
       </c>
       <c r="L179" s="4" t="n">
         <f aca="false">I179*J179</f>
-        <v>0.036</v>
+        <v>0.1656</v>
       </c>
       <c r="M179" s="4" t="n">
         <f aca="false">MIN(1,I179*J179*K179)</f>
-        <v>0.054</v>
+        <v>0.2484</v>
       </c>
       <c r="N179" s="4" t="n">
         <f aca="false">N178*M179</f>
-        <v>0.007776</v>
+        <v>0.0357696</v>
       </c>
       <c r="O179" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -20449,7 +20449,7 @@
       </c>
       <c r="AA179" s="3" t="n">
         <f aca="false">IF(J179&gt;='Settings '!$B$10,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB179" s="3" t="n">
         <f aca="false">IF(M179&gt;='Settings '!$B$11,1,0)</f>
@@ -20504,7 +20504,7 @@
       </c>
       <c r="N180" s="4" t="n">
         <f aca="false">N179*M180</f>
-        <v>0.000559872</v>
+        <v>0.0025754112</v>
       </c>
       <c r="O180" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -20611,7 +20611,7 @@
       </c>
       <c r="N181" s="4" t="n">
         <f aca="false">N180*M181</f>
-        <v>0.00010077696</v>
+        <v>0.000463574016</v>
       </c>
       <c r="O181" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -20639,7 +20639,7 @@
       </c>
       <c r="U181" s="4" t="n">
         <f aca="false">IF(E181=4,N181,"")</f>
-        <v>0.00010077696</v>
+        <v>0.000463574016</v>
       </c>
       <c r="V181" s="4" t="n">
         <f aca="false">IF(E181=4,Q181,"")</f>
@@ -20651,7 +20651,7 @@
       </c>
       <c r="X181" s="4" t="n">
         <f aca="false">IF(E181=4,IFERROR((LN(U181)-LN(V181))/(LN(W181)-LN(V181)),0),"")</f>
-        <v>0</v>
+        <v>0.189638418693276</v>
       </c>
       <c r="Y181" s="3" t="str">
         <f aca="false">IF(E181=4,IF(X181&gt;='Settings '!$B$7,"Risk A",IF(X181&gt;='Settings '!$B$6,"Risk B","Risk C")),"")</f>
@@ -20810,22 +20810,22 @@
         <v>0.36</v>
       </c>
       <c r="J183" s="4" t="n">
-        <v>0.1</v>
+        <v>0.46</v>
       </c>
       <c r="K183" s="4" t="n">
         <v>1.5</v>
       </c>
       <c r="L183" s="4" t="n">
         <f aca="false">I183*J183</f>
-        <v>0.036</v>
+        <v>0.1656</v>
       </c>
       <c r="M183" s="4" t="n">
         <f aca="false">MIN(1,I183*J183*K183)</f>
-        <v>0.054</v>
+        <v>0.2484</v>
       </c>
       <c r="N183" s="4" t="n">
         <f aca="false">N182*M183</f>
-        <v>0.007776</v>
+        <v>0.0357696</v>
       </c>
       <c r="O183" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -20877,7 +20877,7 @@
       </c>
       <c r="AA183" s="3" t="n">
         <f aca="false">IF(J183&gt;='Settings '!$B$10,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB183" s="3" t="n">
         <f aca="false">IF(M183&gt;='Settings '!$B$11,1,0)</f>
@@ -20932,7 +20932,7 @@
       </c>
       <c r="N184" s="4" t="n">
         <f aca="false">N183*M184</f>
-        <v>0.000559872</v>
+        <v>0.0025754112</v>
       </c>
       <c r="O184" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -21039,7 +21039,7 @@
       </c>
       <c r="N185" s="4" t="n">
         <f aca="false">N184*M185</f>
-        <v>0.0002257403904</v>
+        <v>0.00103840579584</v>
       </c>
       <c r="O185" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -21067,7 +21067,7 @@
       </c>
       <c r="U185" s="4" t="n">
         <f aca="false">IF(E185=4,N185,"")</f>
-        <v>0.0002257403904</v>
+        <v>0.00103840579584</v>
       </c>
       <c r="V185" s="4" t="n">
         <f aca="false">IF(E185=4,Q185,"")</f>
@@ -21079,7 +21079,7 @@
       </c>
       <c r="X185" s="4" t="n">
         <f aca="false">IF(E185=4,IFERROR((LN(U185)-LN(V185))/(LN(W185)-LN(V185)),0),"")</f>
-        <v>0.124495519473378</v>
+        <v>0.309017265158183</v>
       </c>
       <c r="Y185" s="3" t="str">
         <f aca="false">IF(E185=4,IF(X185&gt;='Settings '!$B$7,"Risk A",IF(X185&gt;='Settings '!$B$6,"Risk B","Risk C")),"")</f>
@@ -21238,22 +21238,22 @@
         <v>0.36</v>
       </c>
       <c r="J187" s="4" t="n">
-        <v>0.1</v>
+        <v>0.46</v>
       </c>
       <c r="K187" s="4" t="n">
         <v>1.5</v>
       </c>
       <c r="L187" s="4" t="n">
         <f aca="false">I187*J187</f>
-        <v>0.036</v>
+        <v>0.1656</v>
       </c>
       <c r="M187" s="4" t="n">
         <f aca="false">MIN(1,I187*J187*K187)</f>
-        <v>0.054</v>
+        <v>0.2484</v>
       </c>
       <c r="N187" s="4" t="n">
         <f aca="false">N186*M187</f>
-        <v>0.007776</v>
+        <v>0.0357696</v>
       </c>
       <c r="O187" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -21305,7 +21305,7 @@
       </c>
       <c r="AA187" s="3" t="n">
         <f aca="false">IF(J187&gt;='Settings '!$B$10,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB187" s="3" t="n">
         <f aca="false">IF(M187&gt;='Settings '!$B$11,1,0)</f>
@@ -21360,7 +21360,7 @@
       </c>
       <c r="N188" s="4" t="n">
         <f aca="false">N187*M188</f>
-        <v>0.000559872</v>
+        <v>0.0025754112</v>
       </c>
       <c r="O188" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -21467,7 +21467,7 @@
       </c>
       <c r="N189" s="4" t="n">
         <f aca="false">N188*M189</f>
-        <v>5.64350976E-005</v>
+        <v>0.00025960144896</v>
       </c>
       <c r="O189" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -21495,7 +21495,7 @@
       </c>
       <c r="U189" s="4" t="n">
         <f aca="false">IF(E189=4,N189,"")</f>
-        <v>5.64350976E-005</v>
+        <v>0.00025960144896</v>
       </c>
       <c r="V189" s="4" t="n">
         <f aca="false">IF(E189=4,Q189,"")</f>
@@ -21507,7 +21507,7 @@
       </c>
       <c r="X189" s="4" t="n">
         <f aca="false">IF(E189=4,IFERROR((LN(U189)-LN(V189))/(LN(W189)-LN(V189)),0),"")</f>
-        <v>0.120711114312368</v>
+        <v>0.29962378225974</v>
       </c>
       <c r="Y189" s="3" t="str">
         <f aca="false">IF(E189=4,IF(X189&gt;='Settings '!$B$7,"Risk A",IF(X189&gt;='Settings '!$B$6,"Risk B","Risk C")),"")</f>
@@ -21666,22 +21666,22 @@
         <v>0.36</v>
       </c>
       <c r="J191" s="4" t="n">
-        <v>0.1</v>
+        <v>0.46</v>
       </c>
       <c r="K191" s="4" t="n">
         <v>1.5</v>
       </c>
       <c r="L191" s="4" t="n">
         <f aca="false">I191*J191</f>
-        <v>0.036</v>
+        <v>0.1656</v>
       </c>
       <c r="M191" s="4" t="n">
         <f aca="false">MIN(1,I191*J191*K191)</f>
-        <v>0.054</v>
+        <v>0.2484</v>
       </c>
       <c r="N191" s="4" t="n">
         <f aca="false">N190*M191</f>
-        <v>0.007776</v>
+        <v>0.0357696</v>
       </c>
       <c r="O191" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -21733,7 +21733,7 @@
       </c>
       <c r="AA191" s="3" t="n">
         <f aca="false">IF(J191&gt;='Settings '!$B$10,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB191" s="3" t="n">
         <f aca="false">IF(M191&gt;='Settings '!$B$11,1,0)</f>
@@ -21788,7 +21788,7 @@
       </c>
       <c r="N192" s="4" t="n">
         <f aca="false">N191*M192</f>
-        <v>0.000559872</v>
+        <v>0.0025754112</v>
       </c>
       <c r="O192" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -21895,7 +21895,7 @@
       </c>
       <c r="N193" s="4" t="n">
         <f aca="false">N192*M193</f>
-        <v>5.64350976E-005</v>
+        <v>0.00025960144896</v>
       </c>
       <c r="O193" s="4" t="n">
         <f aca="false">'Settings '!$B$8</f>
@@ -21923,7 +21923,7 @@
       </c>
       <c r="U193" s="4" t="n">
         <f aca="false">IF(E193=4,N193,"")</f>
-        <v>5.64350976E-005</v>
+        <v>0.00025960144896</v>
       </c>
       <c r="V193" s="4" t="n">
         <f aca="false">IF(E193=4,Q193,"")</f>
@@ -21935,7 +21935,7 @@
       </c>
       <c r="X193" s="4" t="n">
         <f aca="false">IF(E193=4,IFERROR((LN(U193)-LN(V193))/(LN(W193)-LN(V193)),0),"")</f>
-        <v>0.120711114312368</v>
+        <v>0.29962378225974</v>
       </c>
       <c r="Y193" s="3" t="str">
         <f aca="false">IF(E193=4,IF(X193&gt;='Settings '!$B$7,"Risk A",IF(X193&gt;='Settings '!$B$6,"Risk B","Risk C")),"")</f>
@@ -28827,7 +28827,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L65"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14"/>
@@ -30309,7 +30309,7 @@
       </c>
       <c r="E34" s="4" t="n">
         <f aca="false">LONG!U133</f>
-        <v>0.00010077696</v>
+        <v>0.000463574016</v>
       </c>
       <c r="F34" s="4" t="n">
         <f aca="false">LONG!V133</f>
@@ -30321,7 +30321,7 @@
       </c>
       <c r="H34" s="4" t="n">
         <f aca="false">LONG!X133</f>
-        <v>0</v>
+        <v>0.189638418693276</v>
       </c>
       <c r="I34" s="3" t="str">
         <f aca="false">LONG!Y133</f>
@@ -30353,7 +30353,7 @@
       </c>
       <c r="E35" s="4" t="n">
         <f aca="false">LONG!U137</f>
-        <v>0.0002257403904</v>
+        <v>0.00103840579584</v>
       </c>
       <c r="F35" s="4" t="n">
         <f aca="false">LONG!V137</f>
@@ -30365,7 +30365,7 @@
       </c>
       <c r="H35" s="4" t="n">
         <f aca="false">LONG!X137</f>
-        <v>0.124495519473378</v>
+        <v>0.309017265158183</v>
       </c>
       <c r="I35" s="3" t="str">
         <f aca="false">LONG!Y137</f>
@@ -30397,7 +30397,7 @@
       </c>
       <c r="E36" s="4" t="n">
         <f aca="false">LONG!U141</f>
-        <v>5.64350976E-005</v>
+        <v>0.00025960144896</v>
       </c>
       <c r="F36" s="4" t="n">
         <f aca="false">LONG!V141</f>
@@ -30409,7 +30409,7 @@
       </c>
       <c r="H36" s="4" t="n">
         <f aca="false">LONG!X141</f>
-        <v>0.120711114312368</v>
+        <v>0.29962378225974</v>
       </c>
       <c r="I36" s="3" t="str">
         <f aca="false">LONG!Y141</f>
@@ -30441,7 +30441,7 @@
       </c>
       <c r="E37" s="4" t="n">
         <f aca="false">LONG!U145</f>
-        <v>5.64350976E-005</v>
+        <v>0.00025960144896</v>
       </c>
       <c r="F37" s="4" t="n">
         <f aca="false">LONG!V145</f>
@@ -30453,7 +30453,7 @@
       </c>
       <c r="H37" s="4" t="n">
         <f aca="false">LONG!X145</f>
-        <v>0.120711114312368</v>
+        <v>0.29962378225974</v>
       </c>
       <c r="I37" s="3" t="str">
         <f aca="false">LONG!Y145</f>
@@ -30485,7 +30485,7 @@
       </c>
       <c r="E38" s="4" t="n">
         <f aca="false">LONG!U149</f>
-        <v>0.00010077696</v>
+        <v>0.000463574016</v>
       </c>
       <c r="F38" s="4" t="n">
         <f aca="false">LONG!V149</f>
@@ -30497,7 +30497,7 @@
       </c>
       <c r="H38" s="4" t="n">
         <f aca="false">LONG!X149</f>
-        <v>0</v>
+        <v>0.189638418693276</v>
       </c>
       <c r="I38" s="3" t="str">
         <f aca="false">LONG!Y149</f>
@@ -30529,7 +30529,7 @@
       </c>
       <c r="E39" s="4" t="n">
         <f aca="false">LONG!U153</f>
-        <v>0.0002257403904</v>
+        <v>0.00103840579584</v>
       </c>
       <c r="F39" s="4" t="n">
         <f aca="false">LONG!V153</f>
@@ -30541,7 +30541,7 @@
       </c>
       <c r="H39" s="4" t="n">
         <f aca="false">LONG!X153</f>
-        <v>0.124495519473378</v>
+        <v>0.309017265158183</v>
       </c>
       <c r="I39" s="3" t="str">
         <f aca="false">LONG!Y153</f>
@@ -30573,7 +30573,7 @@
       </c>
       <c r="E40" s="4" t="n">
         <f aca="false">LONG!U157</f>
-        <v>5.64350976E-005</v>
+        <v>0.00025960144896</v>
       </c>
       <c r="F40" s="4" t="n">
         <f aca="false">LONG!V157</f>
@@ -30585,7 +30585,7 @@
       </c>
       <c r="H40" s="4" t="n">
         <f aca="false">LONG!X157</f>
-        <v>0.120711114312368</v>
+        <v>0.29962378225974</v>
       </c>
       <c r="I40" s="3" t="str">
         <f aca="false">LONG!Y157</f>
@@ -30617,7 +30617,7 @@
       </c>
       <c r="E41" s="4" t="n">
         <f aca="false">LONG!U161</f>
-        <v>5.64350976E-005</v>
+        <v>0.00025960144896</v>
       </c>
       <c r="F41" s="4" t="n">
         <f aca="false">LONG!V161</f>
@@ -30629,7 +30629,7 @@
       </c>
       <c r="H41" s="4" t="n">
         <f aca="false">LONG!X161</f>
-        <v>0.120711114312368</v>
+        <v>0.29962378225974</v>
       </c>
       <c r="I41" s="3" t="str">
         <f aca="false">LONG!Y161</f>
@@ -30661,7 +30661,7 @@
       </c>
       <c r="E42" s="4" t="n">
         <f aca="false">LONG!U165</f>
-        <v>0.00010077696</v>
+        <v>0.000463574016</v>
       </c>
       <c r="F42" s="4" t="n">
         <f aca="false">LONG!V165</f>
@@ -30673,7 +30673,7 @@
       </c>
       <c r="H42" s="4" t="n">
         <f aca="false">LONG!X165</f>
-        <v>0</v>
+        <v>0.189638418693276</v>
       </c>
       <c r="I42" s="3" t="str">
         <f aca="false">LONG!Y165</f>
@@ -30705,7 +30705,7 @@
       </c>
       <c r="E43" s="4" t="n">
         <f aca="false">LONG!U169</f>
-        <v>0.0002257403904</v>
+        <v>0.00103840579584</v>
       </c>
       <c r="F43" s="4" t="n">
         <f aca="false">LONG!V169</f>
@@ -30717,7 +30717,7 @@
       </c>
       <c r="H43" s="4" t="n">
         <f aca="false">LONG!X169</f>
-        <v>0.124495519473378</v>
+        <v>0.309017265158183</v>
       </c>
       <c r="I43" s="3" t="str">
         <f aca="false">LONG!Y169</f>
@@ -30749,7 +30749,7 @@
       </c>
       <c r="E44" s="4" t="n">
         <f aca="false">LONG!U173</f>
-        <v>5.64350976E-005</v>
+        <v>0.00025960144896</v>
       </c>
       <c r="F44" s="4" t="n">
         <f aca="false">LONG!V173</f>
@@ -30761,7 +30761,7 @@
       </c>
       <c r="H44" s="4" t="n">
         <f aca="false">LONG!X173</f>
-        <v>0.120711114312368</v>
+        <v>0.29962378225974</v>
       </c>
       <c r="I44" s="3" t="str">
         <f aca="false">LONG!Y173</f>
@@ -30793,7 +30793,7 @@
       </c>
       <c r="E45" s="4" t="n">
         <f aca="false">LONG!U177</f>
-        <v>5.64350976E-005</v>
+        <v>0.00025960144896</v>
       </c>
       <c r="F45" s="4" t="n">
         <f aca="false">LONG!V177</f>
@@ -30805,7 +30805,7 @@
       </c>
       <c r="H45" s="4" t="n">
         <f aca="false">LONG!X177</f>
-        <v>0.120711114312368</v>
+        <v>0.29962378225974</v>
       </c>
       <c r="I45" s="3" t="str">
         <f aca="false">LONG!Y177</f>
@@ -30837,7 +30837,7 @@
       </c>
       <c r="E46" s="4" t="n">
         <f aca="false">LONG!U181</f>
-        <v>0.00010077696</v>
+        <v>0.000463574016</v>
       </c>
       <c r="F46" s="4" t="n">
         <f aca="false">LONG!V181</f>
@@ -30849,7 +30849,7 @@
       </c>
       <c r="H46" s="4" t="n">
         <f aca="false">LONG!X181</f>
-        <v>0</v>
+        <v>0.189638418693276</v>
       </c>
       <c r="I46" s="3" t="str">
         <f aca="false">LONG!Y181</f>
@@ -30881,7 +30881,7 @@
       </c>
       <c r="E47" s="4" t="n">
         <f aca="false">LONG!U185</f>
-        <v>0.0002257403904</v>
+        <v>0.00103840579584</v>
       </c>
       <c r="F47" s="4" t="n">
         <f aca="false">LONG!V185</f>
@@ -30893,7 +30893,7 @@
       </c>
       <c r="H47" s="4" t="n">
         <f aca="false">LONG!X185</f>
-        <v>0.124495519473378</v>
+        <v>0.309017265158183</v>
       </c>
       <c r="I47" s="3" t="str">
         <f aca="false">LONG!Y185</f>
@@ -30925,7 +30925,7 @@
       </c>
       <c r="E48" s="4" t="n">
         <f aca="false">LONG!U189</f>
-        <v>5.64350976E-005</v>
+        <v>0.00025960144896</v>
       </c>
       <c r="F48" s="4" t="n">
         <f aca="false">LONG!V189</f>
@@ -30937,7 +30937,7 @@
       </c>
       <c r="H48" s="4" t="n">
         <f aca="false">LONG!X189</f>
-        <v>0.120711114312368</v>
+        <v>0.29962378225974</v>
       </c>
       <c r="I48" s="3" t="str">
         <f aca="false">LONG!Y189</f>
@@ -30969,7 +30969,7 @@
       </c>
       <c r="E49" s="4" t="n">
         <f aca="false">LONG!U193</f>
-        <v>5.64350976E-005</v>
+        <v>0.00025960144896</v>
       </c>
       <c r="F49" s="4" t="n">
         <f aca="false">LONG!V193</f>
@@ -30981,7 +30981,7 @@
       </c>
       <c r="H49" s="4" t="n">
         <f aca="false">LONG!X193</f>
-        <v>0.120711114312368</v>
+        <v>0.29962378225974</v>
       </c>
       <c r="I49" s="3" t="str">
         <f aca="false">LONG!Y193</f>
@@ -31722,7 +31722,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24"/>
@@ -31787,7 +31787,7 @@
       </c>
       <c r="B7" s="7" t="n">
         <f aca="false">MAX(Tree_Summary!E2:E65)</f>
-        <v>0.00031603654656</v>
+        <v>0.00103840579584</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -31796,7 +31796,7 @@
       </c>
       <c r="B8" s="1" t="str">
         <f aca="false">INDEX(Tree_Summary!C2:C65,MATCH(B7,Tree_Summary!E2:E65,0))</f>
-        <v>A-050</v>
+        <v>A-034</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -31805,7 +31805,7 @@
       </c>
       <c r="B9" s="7" t="n">
         <f aca="false">AVERAGE(Tree_Summary!E2:E65)</f>
-        <v>0.00012083157504</v>
+        <v>0.0002196937728</v>
       </c>
     </row>
   </sheetData>
@@ -31825,7 +31825,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D19"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
@@ -32058,7 +32058,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="90"/>

</xml_diff>